<commit_message>
Restructure source data files
</commit_message>
<xml_diff>
--- a/GPS-Speedsurfing_Equipment_Cleanup.xlsx
+++ b/GPS-Speedsurfing_Equipment_Cleanup.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bjorn\Documents\bjorn76\WS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD7D76E0-D3A5-4FBF-8F92-160276309F14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{055A99B7-C54B-4522-BC15-7C35A341DBD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6090" yWindow="5580" windowWidth="28410" windowHeight="14910" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Systematic" sheetId="1" r:id="rId1"/>
-    <sheet name="Ad-hoc" sheetId="2" r:id="rId2"/>
+    <sheet name="Boards_Status" sheetId="3" r:id="rId1"/>
+    <sheet name="Sails_Status" sheetId="1" r:id="rId2"/>
+    <sheet name="Ad-hoc" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="32">
   <si>
     <t>Year</t>
   </si>
@@ -87,17 +88,103 @@
     <t>Fanatic</t>
   </si>
   <si>
-    <t>Date Started</t>
-  </si>
-  <si>
-    <t>Date Completed</t>
+    <t>Falcons data is missing</t>
+  </si>
+  <si>
+    <t>CSV</t>
+  </si>
+  <si>
+    <t>2007_Fanatic.pdf</t>
+  </si>
+  <si>
+    <t>2010_Fanatic.pdf</t>
+  </si>
+  <si>
+    <t>2016_Fanatic.pdf</t>
+  </si>
+  <si>
+    <t>2018_Fanatic.pdf</t>
+  </si>
+  <si>
+    <t>2020_Fanatic.pdf</t>
+  </si>
+  <si>
+    <t>2007_Fanatic.csv</t>
+  </si>
+  <si>
+    <t>2010_Fanatic.csv</t>
+  </si>
+  <si>
+    <t>2016_Fanatic.csv</t>
+  </si>
+  <si>
+    <t>2020_Fanatic.csv</t>
+  </si>
+  <si>
+    <t>Data Source</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>pdf/picture</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Date added to</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Board Ref.
+Catalogue</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Date when </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Quick Cleaned</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -113,16 +200,56 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -130,14 +257,41 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -417,44 +571,360 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C839D74-D0CF-408E-948F-CB970C57D641}">
+  <dimension ref="A1:H19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.7109375" customWidth="1"/>
+    <col min="3" max="3" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.140625" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21" customWidth="1"/>
+    <col min="8" max="8" width="34.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:8" ht="21" x14ac:dyDescent="0.35">
+      <c r="D1" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="3"/>
+    </row>
+    <row r="2" spans="1:8" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D2" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="4">
+        <v>1</v>
+      </c>
+      <c r="B3" s="4">
+        <v>2007</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F3" s="9">
+        <v>46132</v>
+      </c>
+      <c r="G3" s="8"/>
+      <c r="H3" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="E1" t="s">
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="4">
+        <v>2</v>
+      </c>
+      <c r="B4" s="4">
+        <v>2008</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="5"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="8"/>
+      <c r="H4" s="7"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="4">
+        <v>3</v>
+      </c>
+      <c r="B5" s="4">
+        <v>2009</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="5"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="7"/>
+      <c r="G5" s="8"/>
+      <c r="H5" s="7"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="4">
+        <v>4</v>
+      </c>
+      <c r="B6" s="4">
+        <v>2010</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="F6" s="9">
+        <v>46132</v>
+      </c>
+      <c r="G6" s="8"/>
+      <c r="H6" s="7"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="4">
+        <v>5</v>
+      </c>
+      <c r="B7" s="4">
+        <v>2011</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" s="5"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="7"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="7"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="4">
+        <v>6</v>
+      </c>
+      <c r="B8" s="4">
+        <v>2012</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D8" s="5"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="7"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="4">
+        <v>7</v>
+      </c>
+      <c r="B9" s="4">
+        <v>2013</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9" s="5"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="7"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" s="4">
+        <v>8</v>
+      </c>
+      <c r="B10" s="4">
+        <v>2014</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D10" s="5"/>
+      <c r="E10" s="6"/>
+      <c r="F10" s="7"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="7"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" s="4">
+        <v>9</v>
+      </c>
+      <c r="B11" s="4">
+        <v>2015</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D11" s="5"/>
+      <c r="E11" s="6"/>
+      <c r="F11" s="7"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="7"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" s="4">
+        <v>10</v>
+      </c>
+      <c r="B12" s="4">
+        <v>2016</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F12" s="9">
+        <v>46131</v>
+      </c>
+      <c r="G12" s="8"/>
+      <c r="H12" s="7"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="4">
+        <v>11</v>
+      </c>
+      <c r="B13" s="4">
+        <v>2017</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D13" s="5"/>
+      <c r="E13" s="6"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="7"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" s="4">
+        <v>12</v>
+      </c>
+      <c r="B14" s="4">
+        <v>2018</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F14" s="9">
+        <v>46131</v>
+      </c>
+      <c r="G14" s="8"/>
+      <c r="H14" s="7"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="4">
+        <v>13</v>
+      </c>
+      <c r="B15" s="4">
+        <v>2019</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D15" s="5"/>
+      <c r="E15" s="6"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="7"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="4">
+        <v>14</v>
+      </c>
+      <c r="B16" s="4">
+        <v>2020</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D16" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="F16" s="9">
+        <v>46132</v>
+      </c>
+      <c r="G16" s="8"/>
+      <c r="H16" s="7"/>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" s="4">
+        <v>15</v>
+      </c>
+      <c r="B17" s="4">
+        <v>2021</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D17" s="5"/>
+      <c r="E17" s="6"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="7"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" s="4">
+        <v>16</v>
+      </c>
+      <c r="B18" s="4">
+        <v>2022</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D18" s="5"/>
+      <c r="E18" s="6"/>
+      <c r="F18" s="7"/>
+      <c r="G18" s="8"/>
+      <c r="H18" s="7"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="4">
         <v>17</v>
       </c>
-      <c r="F1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>2018</v>
-      </c>
-      <c r="C2" t="s">
-        <v>15</v>
-      </c>
+      <c r="B19" s="4">
+        <v>2023</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="F19" s="9">
+        <v>46131</v>
+      </c>
+      <c r="G19" s="8"/>
+      <c r="H19" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -462,107 +932,479 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31E37247-C44A-4321-8C2E-00ADA2F53C0B}">
-  <dimension ref="A1:F5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:H19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="6.7109375" customWidth="1"/>
+    <col min="3" max="3" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.140625" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21" customWidth="1"/>
+    <col min="8" max="8" width="34.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="21" x14ac:dyDescent="0.35">
+      <c r="D1" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="3"/>
+    </row>
+    <row r="2" spans="1:8" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="4">
+        <v>1</v>
+      </c>
+      <c r="B3" s="4">
+        <v>2021</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" s="5"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="8"/>
+      <c r="H3" s="7"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="4">
+        <v>2</v>
+      </c>
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="8"/>
+      <c r="H4" s="7"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="4">
+        <v>3</v>
+      </c>
+      <c r="B5" s="4"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="7"/>
+      <c r="G5" s="8"/>
+      <c r="H5" s="7"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="4">
+        <v>4</v>
+      </c>
+      <c r="B6" s="4"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="6"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="7"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="4">
+        <v>5</v>
+      </c>
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="7"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="7"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="4">
+        <v>6</v>
+      </c>
+      <c r="B8" s="4"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="7"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="4">
+        <v>7</v>
+      </c>
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="7"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" s="4">
+        <v>8</v>
+      </c>
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="6"/>
+      <c r="F10" s="7"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="7"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" s="4">
+        <v>9</v>
+      </c>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="6"/>
+      <c r="F11" s="7"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="7"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" s="4">
+        <v>10</v>
+      </c>
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="9"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="7"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="4">
+        <v>11</v>
+      </c>
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="6"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="7"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" s="4">
+        <v>12</v>
+      </c>
+      <c r="B14" s="4"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="7"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="4">
+        <v>13</v>
+      </c>
+      <c r="B15" s="4"/>
+      <c r="C15" s="4"/>
+      <c r="D15" s="5"/>
+      <c r="E15" s="6"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="7"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="4">
+        <v>14</v>
+      </c>
+      <c r="B16" s="4"/>
+      <c r="C16" s="4"/>
+      <c r="D16" s="10"/>
+      <c r="E16" s="6"/>
+      <c r="F16" s="9"/>
+      <c r="G16" s="8"/>
+      <c r="H16" s="7"/>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" s="4">
+        <v>15</v>
+      </c>
+      <c r="B17" s="4"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="6"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="7"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" s="4">
+        <v>16</v>
+      </c>
+      <c r="B18" s="4"/>
+      <c r="C18" s="4"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="6"/>
+      <c r="F18" s="7"/>
+      <c r="G18" s="8"/>
+      <c r="H18" s="7"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="4">
+        <v>17</v>
+      </c>
+      <c r="B19" s="4"/>
+      <c r="C19" s="4"/>
+      <c r="D19" s="5"/>
+      <c r="E19" s="6"/>
+      <c r="F19" s="9"/>
+      <c r="G19" s="8"/>
+      <c r="H19" s="7"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31E37247-C44A-4321-8C2E-00ADA2F53C0B}">
+  <dimension ref="A1:F16"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="7" customWidth="1"/>
     <col min="5" max="5" width="10.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="37.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2">
+      <c r="A2" s="4">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="4">
         <v>2020</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="4">
         <v>74</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="11">
         <v>46131</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="4" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3">
+      <c r="A3" s="4">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="4">
         <v>2021</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="11">
         <v>46131</v>
       </c>
+      <c r="F3" s="4"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4">
+      <c r="A4" s="4">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="4">
         <v>2021</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="11">
         <v>46131</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="4" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5">
+      <c r="A5" s="4">
         <v>4</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C5">
+      <c r="C5" s="4">
         <v>2018</v>
       </c>
-      <c r="E5" s="1">
+      <c r="D5" s="4"/>
+      <c r="E5" s="11">
         <v>46131</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="4" t="s">
         <v>13</v>
       </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="4">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="4">
+        <v>6</v>
+      </c>
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="4"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="4">
+        <v>7</v>
+      </c>
+      <c r="B8" s="4"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="4"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="4">
+        <v>8</v>
+      </c>
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="4"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="4">
+        <v>9</v>
+      </c>
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="4"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="4">
+        <v>10</v>
+      </c>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="4">
+        <v>11</v>
+      </c>
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="4"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="4">
+        <v>12</v>
+      </c>
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="4">
+        <v>13</v>
+      </c>
+      <c r="B14" s="4"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
+      <c r="F14" s="4"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="4">
+        <v>14</v>
+      </c>
+      <c r="B15" s="4"/>
+      <c r="C15" s="4"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+      <c r="F15" s="4"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="4">
+        <v>15</v>
+      </c>
+      <c r="B16" s="4"/>
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
+      <c r="F16" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>